<commit_message>
Updated Basic Practise File.xlsx
</commit_message>
<xml_diff>
--- a/Basic Operations/Basic Practise File.xlsx
+++ b/Basic Operations/Basic Practise File.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\Basic Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA7CA01B-DADB-495A-974D-81796C51211E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F102F5D3-8CA0-45F1-BFE7-8412597D1DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="955" firstSheet="6" activeTab="13" xr2:uid="{804A284F-30AB-4AA4-80D9-3863464D9C5B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="955" firstSheet="6" activeTab="6" xr2:uid="{804A284F-30AB-4AA4-80D9-3863464D9C5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="13" r:id="rId1"/>
@@ -345,9 +345,6 @@
     <t>SQRT</t>
   </si>
   <si>
-    <t>Emp Code</t>
-  </si>
-  <si>
     <t>Address</t>
   </si>
   <si>
@@ -1396,6 +1393,9 @@
   </si>
   <si>
     <t>then click finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1803,7 +1803,7 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -1811,7 +1811,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1819,7 +1819,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1827,7 +1827,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -1835,7 +1835,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -1843,7 +1843,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -1851,7 +1851,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -1859,7 +1859,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -1867,7 +1867,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -1875,7 +1875,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -1883,7 +1883,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -1891,7 +1891,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -1899,7 +1899,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -1907,7 +1907,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -1915,7 +1915,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -1923,7 +1923,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1931,7 +1931,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1939,7 +1939,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -1947,7 +1947,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1955,7 +1955,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -1963,7 +1963,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -1971,7 +1971,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -1979,7 +1979,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
@@ -1987,7 +1987,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
@@ -1995,7 +1995,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
@@ -2003,7 +2003,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -2011,7 +2011,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
@@ -2019,7 +2019,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -2027,7 +2027,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -2065,7 +2065,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -2078,13 +2078,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B3">
         <v>12000</v>
       </c>
       <c r="E3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F3">
         <f>SUM(salary)</f>
@@ -2093,13 +2093,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B4">
         <v>11250</v>
       </c>
       <c r="E4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F4">
         <f>AVERAGE(salary)</f>
@@ -2118,7 +2118,7 @@
         <v>12000</v>
       </c>
       <c r="E5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F5">
         <f>MAX(salary)</f>
@@ -2133,7 +2133,7 @@
         <v>16250</v>
       </c>
       <c r="E6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F6">
         <f>MIN(salary)</f>
@@ -2142,13 +2142,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B7">
         <v>6400</v>
       </c>
       <c r="E7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F7">
         <f>COUNT(salary)</f>
@@ -2173,7 +2173,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B10">
         <v>6250</v>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B13">
         <v>10000</v>
@@ -2213,47 +2213,47 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="17" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D19" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D20" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="21" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D21" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="22" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D22" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23" spans="4:6" x14ac:dyDescent="0.35">
       <c r="D23" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F23" cm="1">
         <f t="array" ref="F23:F35">salary</f>
@@ -2353,24 +2353,24 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F1" t="s">
         <v>180</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>181</v>
-      </c>
-      <c r="G1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C2" s="5">
         <v>46154</v>
@@ -2393,10 +2393,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C3" s="12">
         <v>0.4909722222222222</v>
@@ -2404,52 +2404,52 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C4" s="5">
         <f ca="1">TODAY()</f>
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C5" s="6">
         <f ca="1">NOW()</f>
-        <v>46157.949963310188</v>
+        <v>46162.891482060186</v>
       </c>
       <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C6" s="7">
         <f ca="1">NOW()-TODAY()</f>
-        <v>0.94996331018774072</v>
+        <v>0.89148206018580822</v>
       </c>
       <c r="D6" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" t="s">
         <v>180</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>181</v>
       </c>
-      <c r="F6" t="s">
-        <v>182</v>
-      </c>
       <c r="G6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -2476,27 +2476,27 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E10" t="s">
+        <v>192</v>
+      </c>
+      <c r="F10" t="s">
         <v>193</v>
-      </c>
-      <c r="F10" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D11" s="5">
         <f ca="1">TODAY()</f>
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="E11">
         <f ca="1">WEEKDAY(D11)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F11">
         <f ca="1">WEEKNUM(D11)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2522,31 +2522,31 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C1" t="s">
         <v>237</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>243</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>238</v>
       </c>
-      <c r="D1" t="s">
-        <v>244</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>239</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>240</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J1" t="s">
         <v>241</v>
-      </c>
-      <c r="H1" t="s">
-        <v>193</v>
-      </c>
-      <c r="J1" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -2570,17 +2570,17 @@
       </c>
       <c r="G2" s="5">
         <f ca="1">TODAY()</f>
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="H2" s="5">
         <f ca="1">TODAY()</f>
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="J2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="L2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
@@ -2610,13 +2610,13 @@
         <v>46160</v>
       </c>
       <c r="J3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="L3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="N3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
@@ -2646,16 +2646,16 @@
         <v>46161</v>
       </c>
       <c r="J4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="L4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="N4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="O4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -2685,16 +2685,16 @@
         <v>46162</v>
       </c>
       <c r="J5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="L5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="N5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="O5" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -2724,16 +2724,16 @@
         <v>46163</v>
       </c>
       <c r="J6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="L6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="N6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="O6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -2763,16 +2763,16 @@
         <v>46164</v>
       </c>
       <c r="J7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="L7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="N7" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="O7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -2802,16 +2802,16 @@
         <v>46167</v>
       </c>
       <c r="J8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="L8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="N8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="O8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -2841,16 +2841,16 @@
         <v>46168</v>
       </c>
       <c r="J9" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="L9" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="N9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="O9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
@@ -2877,10 +2877,10 @@
         <v>46169</v>
       </c>
       <c r="J10" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="L10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
@@ -2907,133 +2907,133 @@
         <v>46170</v>
       </c>
       <c r="J11" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="L11" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="L12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="N12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="L13" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="N13" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="N14" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D15" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H15" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J15" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="N15" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E16" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F16" t="s">
+        <v>332</v>
+      </c>
+      <c r="G16" t="s">
         <v>333</v>
       </c>
-      <c r="G16" t="s">
-        <v>334</v>
-      </c>
       <c r="H16" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J16" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="N16" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F17" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G17" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H17" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="N17" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D18" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F18" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H18" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="N18" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.35">
       <c r="N19" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.35">
       <c r="N20" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -3057,28 +3057,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" t="s">
         <v>183</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D1" t="s">
         <v>184</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F1" t="s">
+        <v>186</v>
+      </c>
+      <c r="G1" t="s">
         <v>188</v>
       </c>
-      <c r="D1" t="s">
-        <v>185</v>
-      </c>
-      <c r="E1" t="s">
-        <v>186</v>
-      </c>
-      <c r="F1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G1" t="s">
-        <v>189</v>
-      </c>
       <c r="H1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -3216,7 +3216,7 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <f ca="1">TODAY()</f>
-        <v>46157</v>
+        <v>46162</v>
       </c>
       <c r="B6" t="b">
         <f ca="1"/>
@@ -3232,11 +3232,11 @@
       </c>
       <c r="E6" t="b">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="b">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="b">
         <f t="shared" si="2"/>
@@ -3249,7 +3249,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B7" t="b">
         <f ca="1"/>
@@ -3315,7 +3315,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B9" t="b">
         <f ca="1"/>
@@ -3529,7 +3529,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>0</v>
@@ -3537,16 +3537,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C2">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E2">
         <v>8562</v>
@@ -3560,16 +3560,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E3">
         <v>9845</v>
@@ -3578,44 +3578,44 @@
         <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C4">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E4">
         <v>9878</v>
       </c>
       <c r="F4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G4" t="s">
         <v>396</v>
-      </c>
-      <c r="G4" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C5">
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E5">
         <v>2378</v>
@@ -3627,21 +3627,21 @@
         <v>29</v>
       </c>
       <c r="H5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E6">
         <v>9567</v>
@@ -3650,21 +3650,21 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C7">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E7">
         <v>8923</v>
@@ -3678,16 +3678,16 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B8" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C8">
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E8">
         <v>5679</v>
@@ -3701,16 +3701,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B9" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C9">
         <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E9">
         <v>7453</v>
@@ -3724,16 +3724,16 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C10">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E10">
         <v>4598</v>
@@ -3747,16 +3747,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B11" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E11">
         <v>8345</v>
@@ -3770,94 +3770,94 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C12">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E12">
         <v>3456</v>
       </c>
       <c r="F12" t="s">
+        <v>397</v>
+      </c>
+      <c r="G12" t="s">
         <v>398</v>
-      </c>
-      <c r="G12" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B27" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C27">
         <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E27">
         <v>8562</v>
@@ -3865,16 +3865,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B28" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C28">
         <v>5</v>
       </c>
       <c r="D28" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E28">
         <v>9845</v>
@@ -3882,16 +3882,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B29" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C29">
         <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E29">
         <v>9878</v>
@@ -3899,16 +3899,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B30" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C30">
         <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E30">
         <v>2378</v>
@@ -3916,16 +3916,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B31" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C31">
         <v>4</v>
       </c>
       <c r="D31" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E31">
         <v>9567</v>
@@ -3933,16 +3933,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B32" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C32">
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E32">
         <v>8923</v>
@@ -3950,16 +3950,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C33">
         <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E33">
         <v>5679</v>
@@ -3967,16 +3967,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C34">
         <v>9</v>
       </c>
       <c r="D34" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E34">
         <v>7453</v>
@@ -3984,16 +3984,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B35" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C35">
         <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E35">
         <v>4598</v>
@@ -4001,16 +4001,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B36" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C36">
         <v>3</v>
       </c>
       <c r="D36" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E36">
         <v>8345</v>
@@ -4018,16 +4018,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B37" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C37">
         <v>5</v>
       </c>
       <c r="D37" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E37">
         <v>3456</v>
@@ -4064,10 +4064,10 @@
         <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -4080,13 +4080,13 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F2" s="11"/>
     </row>
@@ -4098,10 +4098,10 @@
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E3" s="11"/>
       <c r="F3" s="11"/>
@@ -4114,10 +4114,10 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
@@ -4130,10 +4130,10 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
@@ -4146,10 +4146,10 @@
         <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
@@ -4162,10 +4162,10 @@
         <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
@@ -4178,10 +4178,10 @@
         <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
@@ -4194,10 +4194,10 @@
         <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="11"/>
@@ -4210,10 +4210,10 @@
         <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
@@ -4226,10 +4226,10 @@
         <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
@@ -4294,10 +4294,10 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
+        <v>270</v>
+      </c>
+      <c r="J1" t="s">
         <v>271</v>
-      </c>
-      <c r="J1" t="s">
-        <v>272</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>41</v>
@@ -4333,7 +4333,7 @@
         <v>50</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>0</v>
@@ -4761,7 +4761,7 @@
         <v>Sanjay GuptA</v>
       </c>
       <c r="N6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="O6" t="s">
         <v>5</v>
@@ -5264,48 +5264,48 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="P13" t="s">
+        <v>272</v>
+      </c>
+      <c r="Q13" t="s">
         <v>273</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="U13" t="s">
         <v>274</v>
-      </c>
-      <c r="U13" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -5536,13 +5536,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
@@ -5626,13 +5626,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
@@ -5656,17 +5656,17 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -5968,49 +5968,49 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" t="s">
         <v>284</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>285</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>286</v>
-      </c>
-      <c r="E11" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H12" t="s">
+        <v>287</v>
+      </c>
+      <c r="I12" t="s">
         <v>288</v>
-      </c>
-      <c r="I12" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f ca="1">RAND()</f>
-        <v>0.29646970589883925</v>
+        <v>4.7847909005719225E-2</v>
       </c>
       <c r="I13" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -6067,7 +6067,7 @@
         <v>67</v>
       </c>
       <c r="J1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K1" t="s">
         <v>56</v>
@@ -6079,7 +6079,7 @@
         <v>56</v>
       </c>
       <c r="O1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="Q1" t="s">
         <v>56</v>
@@ -6100,7 +6100,7 @@
         <v>56</v>
       </c>
       <c r="Y1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.35">
@@ -6718,56 +6718,56 @@
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
+        <v>290</v>
+      </c>
+      <c r="C13" t="s">
         <v>291</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>292</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>293</v>
-      </c>
-      <c r="E13" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
+        <v>294</v>
+      </c>
+      <c r="C14" t="s">
         <v>295</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>296</v>
       </c>
-      <c r="D14" t="s">
+      <c r="I14" t="s">
         <v>297</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>298</v>
       </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
         <v>299</v>
       </c>
-      <c r="L14" t="s">
+      <c r="O14" t="s">
         <v>300</v>
       </c>
-      <c r="O14" t="s">
+      <c r="R14" t="s">
         <v>301</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>302</v>
       </c>
-      <c r="S14" t="s">
+      <c r="V14" t="s">
         <v>303</v>
       </c>
-      <c r="V14" t="s">
+      <c r="Y14" t="s">
         <v>304</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.35">
       <c r="R15" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.35">
@@ -6814,28 +6814,28 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>440</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -6846,16 +6846,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" t="s">
         <v>95</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>96</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>97</v>
-      </c>
-      <c r="F2" t="s">
-        <v>98</v>
       </c>
       <c r="G2" s="3">
         <v>10000</v>
@@ -6873,16 +6873,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" t="s">
         <v>99</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>100</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>101</v>
-      </c>
-      <c r="F3" t="s">
-        <v>102</v>
       </c>
       <c r="G3" s="3">
         <v>12000</v>
@@ -6892,7 +6892,7 @@
         <v>3</v>
       </c>
       <c r="I3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J3" s="3">
         <f>SUM(G2:G21)</f>
@@ -6908,13 +6908,13 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G4" s="3">
         <v>11250</v>
@@ -6924,7 +6924,7 @@
         <v>5</v>
       </c>
       <c r="I4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J4" s="3">
         <f>AVERAGE(G2:G21)</f>
@@ -6940,16 +6940,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
         <v>106</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>107</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>108</v>
-      </c>
-      <c r="F5" t="s">
-        <v>109</v>
       </c>
       <c r="G5" s="3">
         <v>12000</v>
@@ -6959,7 +6959,7 @@
         <v>3</v>
       </c>
       <c r="I5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J5" s="3">
         <f>MAX(G2:G21)</f>
@@ -6975,13 +6975,13 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
         <v>100</v>
       </c>
-      <c r="E6" t="s">
-        <v>101</v>
-      </c>
       <c r="F6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G6" s="3">
         <v>16250</v>
@@ -6991,7 +6991,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J6" s="3">
         <f>MIN(G2:G21)</f>
@@ -7007,16 +7007,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" t="s">
         <v>110</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>111</v>
       </c>
-      <c r="E7" t="s">
-        <v>112</v>
-      </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G7" s="3">
         <v>6400</v>
@@ -7026,7 +7026,7 @@
         <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J7">
         <f>COUNT(G2:G21)</f>
@@ -7041,16 +7041,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" t="s">
         <v>113</v>
       </c>
-      <c r="D8" t="s">
-        <v>114</v>
-      </c>
       <c r="E8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G8" s="3">
         <v>4500</v>
@@ -7060,14 +7060,14 @@
         <v>19</v>
       </c>
       <c r="I8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J8">
         <f>COUNTA(D2:D21)</f>
         <v>19</v>
       </c>
       <c r="L8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M8">
         <f>SUMIFS(G2:G21,F2:F21,F2,E2:E21,E20)</f>
@@ -7082,16 +7082,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G9" s="3">
         <v>6275</v>
@@ -7101,14 +7101,14 @@
         <v>15</v>
       </c>
       <c r="I9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J9">
         <f>COUNTBLANK(C2:C21)</f>
         <v>3</v>
       </c>
       <c r="L9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="M9">
         <f>AVERAGEIFS(G2:G21,F2:F21,F21,E2:E21,E2)</f>
@@ -7123,16 +7123,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D10" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" t="s">
         <v>96</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>97</v>
-      </c>
-      <c r="F10" t="s">
-        <v>98</v>
       </c>
       <c r="G10" s="3">
         <v>6250</v>
@@ -7142,10 +7142,10 @@
         <v>17</v>
       </c>
       <c r="I10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="M10">
         <f>COUNTIFS(F2:F21,F2,E2:E21,E20)</f>
@@ -7160,13 +7160,13 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G11" s="3">
         <v>8750</v>
@@ -7176,7 +7176,7 @@
         <v>11</v>
       </c>
       <c r="I11" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -7184,19 +7184,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" t="s">
         <v>118</v>
       </c>
-      <c r="C12" t="s">
-        <v>119</v>
-      </c>
       <c r="D12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G12" s="3">
         <v>11250</v>
@@ -7206,7 +7206,7 @@
         <v>5</v>
       </c>
       <c r="I12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
@@ -7214,19 +7214,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
         <v>120</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>121</v>
       </c>
-      <c r="D13" t="s">
-        <v>122</v>
-      </c>
       <c r="E13" t="s">
+        <v>107</v>
+      </c>
+      <c r="F13" t="s">
         <v>108</v>
-      </c>
-      <c r="F13" t="s">
-        <v>109</v>
       </c>
       <c r="G13" s="3">
         <v>10000</v>
@@ -7236,7 +7236,7 @@
         <v>8</v>
       </c>
       <c r="I13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
@@ -7244,19 +7244,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" t="s">
         <v>123</v>
       </c>
-      <c r="C14" t="s">
-        <v>99</v>
-      </c>
-      <c r="D14" t="s">
-        <v>124</v>
-      </c>
       <c r="E14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G14" s="3">
         <v>16250</v>
@@ -7266,7 +7266,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -7274,19 +7274,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G15" s="3">
         <v>6400</v>
@@ -7296,10 +7296,10 @@
         <v>13</v>
       </c>
       <c r="I15" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -7307,19 +7307,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" t="s">
         <v>126</v>
       </c>
-      <c r="C16" t="s">
-        <v>127</v>
-      </c>
       <c r="D16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" t="s">
         <v>100</v>
       </c>
-      <c r="E16" t="s">
-        <v>101</v>
-      </c>
       <c r="F16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G16" s="3">
         <v>4500</v>
@@ -7329,10 +7329,10 @@
         <v>19</v>
       </c>
       <c r="I16" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
@@ -7340,16 +7340,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E17" t="s">
+        <v>107</v>
+      </c>
+      <c r="F17" t="s">
         <v>108</v>
-      </c>
-      <c r="F17" t="s">
-        <v>109</v>
       </c>
       <c r="G17" s="3">
         <v>6275</v>
@@ -7359,10 +7359,10 @@
         <v>15</v>
       </c>
       <c r="I17" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -7370,19 +7370,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" t="s">
         <v>129</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" t="s">
         <v>130</v>
-      </c>
-      <c r="D18" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" t="s">
-        <v>97</v>
-      </c>
-      <c r="F18" t="s">
-        <v>131</v>
       </c>
       <c r="G18" s="3">
         <v>6250</v>
@@ -7397,19 +7397,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" t="s">
         <v>132</v>
       </c>
-      <c r="C19" t="s">
-        <v>133</v>
-      </c>
       <c r="D19" t="s">
+        <v>95</v>
+      </c>
+      <c r="E19" t="s">
         <v>96</v>
       </c>
-      <c r="E19" t="s">
-        <v>97</v>
-      </c>
       <c r="F19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G19" s="3">
         <v>8750</v>
@@ -7424,19 +7424,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>133</v>
+      </c>
+      <c r="C20" t="s">
         <v>134</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>135</v>
       </c>
-      <c r="D20" t="s">
-        <v>136</v>
-      </c>
       <c r="E20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G20" s="3">
         <v>11250</v>
@@ -7451,19 +7451,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" t="s">
         <v>137</v>
       </c>
-      <c r="C21" t="s">
-        <v>138</v>
-      </c>
       <c r="D21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G21" s="3">
         <v>10000</v>
@@ -7475,18 +7475,18 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="H24" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="J28" t="s">
+        <v>307</v>
+      </c>
+      <c r="K28" t="s">
         <v>308</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>309</v>
-      </c>
-      <c r="L28" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
@@ -7583,7 +7583,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -7593,12 +7593,12 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B3" s="13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
       <c r="F3" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -7606,30 +7606,30 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" t="s">
         <v>147</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>148</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>149</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>150</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>151</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>152</v>
-      </c>
-      <c r="H4" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B5">
         <v>23</v>
@@ -7642,7 +7642,7 @@
         <v>154.1</v>
       </c>
       <c r="F5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G5">
         <v>8900</v>
@@ -7654,7 +7654,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B6">
         <v>443</v>
@@ -7668,7 +7668,7 @@
       </c>
       <c r="E6" s="5"/>
       <c r="F6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G6">
         <v>45000</v>
@@ -7680,7 +7680,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B7">
         <v>454</v>
@@ -7693,7 +7693,7 @@
         <v>3041.8</v>
       </c>
       <c r="F7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G7">
         <v>34005</v>
@@ -7705,7 +7705,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B8">
         <v>65</v>
@@ -7718,7 +7718,7 @@
         <v>533</v>
       </c>
       <c r="F8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G8">
         <v>23900</v>
@@ -7730,7 +7730,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B9">
         <v>34</v>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="E9" s="5"/>
       <c r="F9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G9">
         <v>32000</v>
@@ -7756,7 +7756,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B10">
         <v>45</v>
@@ -7769,7 +7769,7 @@
         <v>171</v>
       </c>
       <c r="F10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G10">
         <v>12000</v>
@@ -7781,7 +7781,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B11">
         <v>32</v>
@@ -7796,7 +7796,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H13" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -8268,7 +8268,7 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="E16" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="R16">
         <v>10000</v>

</xml_diff>